<commit_message>
Fix typo in FrCorePractitionerRoleCodeCategorieProfessionnelle.fsh 5d865dc88acc7d74aa351db12e16776390c1b650
</commit_message>
<xml_diff>
--- a/nr-add-profile-list/ig/StructureDefinition-fr-core-role-code-categorie-professionnelle.xlsx
+++ b/nr-add-profile-list/ig/StructureDefinition-fr-core-role-code-categorie-professionnelle.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-21T10:59:21+00:00</t>
+    <t>2024-03-21T12:49:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Purpose</t>
   </si>
   <si>
-    <t>Discriminer les étudiants des professionnels de sa,nté diplômés.</t>
+    <t>Discriminer les étudiants des professionnels de santé diplômés.</t>
   </si>
   <si>
     <t>Copyright</t>

</xml_diff>